<commit_message>
Batch 17 shipped: 2026-10-18 stage + five generator features
74 roots shipped (24 new masters, 50 replaced): the 2026-10-18 stage
(OMi answers, Brennan rows marked DimSource BRENNAN, A19-A23, the 37
wrongly-DROP adapters) rebased on the live state after batch 16, built
with the merged hose-barb / flange / angled / per-leg-swivel / straights
features. Generator fix: Atan2V ByVal (angled macros did not compile).
1,354 of 1,874 configurations in a master, 95 masters. Held for
generator work: 4503 4603 1703 1700RC 1800 5404N (QA #175).
RUN_ME_batch17.txt, QA #173-#175, evidence in tools/_out/batch17_20261019.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/04_DESIGN_TABLES/DesignTable_0318.xlsx
+++ b/04_DESIGN_TABLES/DesignTable_0318.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -487,7 +487,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.54</v>
+        <v>0.55</v>
       </c>
       <c r="C3" t="n">
         <v>0.38</v>
@@ -517,7 +517,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Air-Way s47 only (double-pass 13 rows); Air-Way part numbers printed as 318-n; config names zero-padded to 0318-nn</t>
+          <t>Air-Way s47 only (double-pass 13 rows); Air-Way part numbers printed as 318-n; config names zero-padded to 0318-nn; L1@DRIVE: OMi WebsitePartsInfo2026.xlsx Items!L30 = 0.55 (table had 0.54) [user 2026-10-18 A19]</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>A19 (user 2026-10-18, group 3 open): L1@DRIVE 0.54 -&gt; OMi 0.55 (Items!L30, M013)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -538,7 +543,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.6</v>
+        <v>0.61</v>
       </c>
       <c r="C4" t="n">
         <v>0.44</v>
@@ -568,7 +573,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Air-Way s47 only (double-pass 13 rows); Air-Way part numbers printed as 318-n; config names zero-padded to 0318-nn</t>
+          <t>Air-Way s47 only (double-pass 13 rows); Air-Way part numbers printed as 318-n; config names zero-padded to 0318-nn; L1@DRIVE: OMi WebsitePartsInfo2026.xlsx Items!L31 = 0.61 (table had 0.6) [user 2026-10-18 A19]</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>A19 (user 2026-10-18, group 3 open): L1@DRIVE 0.6 -&gt; OMi 0.61 (Items!L31, M013)</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -589,7 +599,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.61</v>
+        <v>0.62</v>
       </c>
       <c r="C5" t="n">
         <v>0.5600000000000001</v>
@@ -619,7 +629,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Air-Way s47 only (double-pass 13 rows); Air-Way part numbers printed as 318-n; config names zero-padded to 0318-nn</t>
+          <t>Air-Way s47 only (double-pass 13 rows); Air-Way part numbers printed as 318-n; config names zero-padded to 0318-nn; L1@DRIVE: OMi WebsitePartsInfo2026.xlsx Items!L32 = 0.62 (table had 0.61) [user 2026-10-18 A19]</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>A19 (user 2026-10-18, group 3 open): L1@DRIVE 0.61 -&gt; OMi 0.62 (Items!L32, M013)</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -640,7 +655,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.67</v>
+        <v>0.68</v>
       </c>
       <c r="C6" t="n">
         <v>0.63</v>
@@ -670,7 +685,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Air-Way s47 only (double-pass 13 rows); Air-Way part numbers printed as 318-n; config names zero-padded to 0318-nn</t>
+          <t>Air-Way s47 only (double-pass 13 rows); Air-Way part numbers printed as 318-n; config names zero-padded to 0318-nn; L1@DRIVE: OMi WebsitePartsInfo2026.xlsx Items!L33 = 0.68 (table had 0.67) [user 2026-10-18 A19]</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>A19 (user 2026-10-18, group 3 open): L1@DRIVE 0.67 -&gt; OMi 0.68 (Items!L33, M013)</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -691,7 +711,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.72</v>
+        <v>0.73</v>
       </c>
       <c r="C7" t="n">
         <v>0.6899999999999999</v>
@@ -721,7 +741,12 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Air-Way s47 only (double-pass 13 rows); Air-Way part numbers printed as 318-n; config names zero-padded to 0318-nn</t>
+          <t>Air-Way s47 only (double-pass 13 rows); Air-Way part numbers printed as 318-n; config names zero-padded to 0318-nn; L1@DRIVE: OMi WebsitePartsInfo2026.xlsx Items!L34 = 0.73 (table had 0.72) [user 2026-10-18 A19]</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>A19 (user 2026-10-18, group 3 open): L1@DRIVE 0.72 -&gt; OMi 0.73 (Items!L34, M013)</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -742,7 +767,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.84</v>
+        <v>0.85</v>
       </c>
       <c r="C8" t="n">
         <v>0.88</v>
@@ -772,7 +797,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Air-Way s47 only (double-pass 13 rows); Air-Way part numbers printed as 318-n; config names zero-padded to 0318-nn</t>
+          <t>Air-Way s47 only (double-pass 13 rows); Air-Way part numbers printed as 318-n; config names zero-padded to 0318-nn; L1@DRIVE: OMi WebsitePartsInfo2026.xlsx Items!L35 = 0.85 (table had 0.84) [user 2026-10-18 A19]</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>A19 (user 2026-10-18, group 3 open): L1@DRIVE 0.84 -&gt; OMi 0.85 (Items!L35, M013)</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -793,7 +823,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.97</v>
+        <v>0.98</v>
       </c>
       <c r="C9" t="n">
         <v>1</v>
@@ -823,7 +853,12 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Air-Way s47 only (double-pass 13 rows); Air-Way part numbers printed as 318-n; config names zero-padded to 0318-nn</t>
+          <t>Air-Way s47 only (double-pass 13 rows); Air-Way part numbers printed as 318-n; config names zero-padded to 0318-nn; L1@DRIVE: OMi WebsitePartsInfo2026.xlsx Items!L36 = 0.98 (table had 0.97) [user 2026-10-18 A19]</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>A19 (user 2026-10-18, group 3 open): L1@DRIVE 0.97 -&gt; OMi 0.98 (Items!L36, M013)</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -844,7 +879,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1.02</v>
+        <v>1.03</v>
       </c>
       <c r="C10" t="n">
         <v>1.25</v>
@@ -874,7 +909,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Air-Way s47 only (double-pass 13 rows); Air-Way part numbers printed as 318-n; config names zero-padded to 0318-nn</t>
+          <t>Air-Way s47 only (double-pass 13 rows); Air-Way part numbers printed as 318-n; config names zero-padded to 0318-nn; L1@DRIVE: OMi WebsitePartsInfo2026.xlsx Items!L37 = 1.03 (table had 1.02) [user 2026-10-18 A19]</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>A19 (user 2026-10-18, group 3 open): L1@DRIVE 1.02 -&gt; OMi 1.03 (Items!L37, M013)</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -946,7 +986,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1.12</v>
+        <v>1.13</v>
       </c>
       <c r="C12" t="n">
         <v>1.5</v>
@@ -976,7 +1016,12 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Air-Way s47 only (double-pass 13 rows); Air-Way part numbers printed as 318-n; config names zero-padded to 0318-nn</t>
+          <t>Air-Way s47 only (double-pass 13 rows); Air-Way part numbers printed as 318-n; config names zero-padded to 0318-nn; L1@DRIVE: OMi WebsitePartsInfo2026.xlsx Items!L38 = 1.13 (table had 1.12) [user 2026-10-18 A19]</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>A19 (user 2026-10-18, group 3 open): L1@DRIVE 1.12 -&gt; OMi 1.13 (Items!L38, M013)</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -997,7 +1042,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1.22</v>
+        <v>1.23</v>
       </c>
       <c r="C13" t="n">
         <v>2</v>
@@ -1027,7 +1072,12 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Air-Way s47 only (double-pass 13 rows); Air-Way part numbers printed as 318-n; config names zero-padded to 0318-nn</t>
+          <t>Air-Way s47 only (double-pass 13 rows); Air-Way part numbers printed as 318-n; config names zero-padded to 0318-nn; L1@DRIVE: OMi WebsitePartsInfo2026.xlsx Items!L39 = 1.23 (table had 1.22) [user 2026-10-18 A19]</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>A19 (user 2026-10-18, group 3 open): L1@DRIVE 1.22 -&gt; OMi 1.23 (Items!L39, M013)</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1073,12 +1123,17 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>ASSUMED</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
           <t>Air-Way s47 only (double-pass 13 rows); Air-Way part numbers printed as 318-n; config names zero-padded to 0318-nn</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>A23 (user 2026-10-18): VERIFIED - OMi = Air-Way on CHEX@HEX=2.25~2.25</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1099,7 +1154,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1.74</v>
+        <v>1.75</v>
       </c>
       <c r="C15" t="n">
         <v>2.88</v>
@@ -1129,7 +1184,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Air-Way s47 only (double-pass 13 rows); Air-Way part numbers printed as 318-n; config names zero-padded to 0318-nn</t>
+          <t>Air-Way s47 only (double-pass 13 rows); Air-Way part numbers printed as 318-n; config names zero-padded to 0318-nn; L1@DRIVE: OMi WebsitePartsInfo2026.xlsx Items!L41 = 1.75 (table had 1.74) [user 2026-10-18 A19]</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>A19 (user 2026-10-18, group 3 open): L1@DRIVE 1.74 -&gt; OMi 1.75 (Items!L41, M013)</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">

</xml_diff>